<commit_message>
updated uploadattendance and submitforapproval ui
</commit_message>
<xml_diff>
--- a/eaas_python/template_files/DTR_template.xlsx
+++ b/eaas_python/template_files/DTR_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Veronica\Downloads\ver\dict_eaas\dict_eeas\backend\template_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Veronica\Downloads\ver\dict_folder\dict_eeas\eaas_python\template_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC6374D-13CD-4253-975B-DB749A443B4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B2CA25-67BD-4034-BFA1-4F2EE57B5D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="24">
   <si>
     <t>CS FORM 48</t>
   </si>
@@ -97,9 +97,6 @@
   </si>
   <si>
     <t>Verified as to Correctness</t>
-  </si>
-  <si>
-    <t>Provincial Officer - Isabela Provincial Office</t>
   </si>
 </sst>
 </file>
@@ -961,15 +958,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -989,6 +992,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -998,28 +1014,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1255,28 +1252,28 @@
     <row r="1" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="84"/>
-      <c r="H3" s="85"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="89"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="90" t="s">
+      <c r="J3" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="84"/>
-      <c r="L3" s="84"/>
-      <c r="M3" s="84"/>
-      <c r="N3" s="84"/>
-      <c r="O3" s="84"/>
-      <c r="P3" s="85"/>
+      <c r="K3" s="88"/>
+      <c r="L3" s="88"/>
+      <c r="M3" s="88"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="88"/>
+      <c r="P3" s="89"/>
     </row>
     <row r="4" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="102" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="79"/>
@@ -1286,7 +1283,7 @@
       <c r="G4" s="79"/>
       <c r="H4" s="80"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="91" t="s">
+      <c r="J4" s="102" t="s">
         <v>1</v>
       </c>
       <c r="K4" s="79"/>
@@ -1315,19 +1312,19 @@
     </row>
     <row r="6" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
-      <c r="C6" s="92"/>
-      <c r="D6" s="77"/>
-      <c r="E6" s="77"/>
-      <c r="F6" s="77"/>
-      <c r="G6" s="77"/>
+      <c r="C6" s="103"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="95"/>
+      <c r="F6" s="95"/>
+      <c r="G6" s="95"/>
       <c r="H6" s="5"/>
       <c r="I6" s="1"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="92"/>
-      <c r="L6" s="77"/>
-      <c r="M6" s="77"/>
-      <c r="N6" s="77"/>
-      <c r="O6" s="77"/>
+      <c r="K6" s="103"/>
+      <c r="L6" s="95"/>
+      <c r="M6" s="95"/>
+      <c r="N6" s="95"/>
+      <c r="O6" s="95"/>
       <c r="P6" s="5"/>
     </row>
     <row r="7" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1353,9 +1350,9 @@
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="77"/>
-      <c r="G8" s="77"/>
+      <c r="E8" s="94"/>
+      <c r="F8" s="95"/>
+      <c r="G8" s="95"/>
       <c r="H8" s="8"/>
       <c r="I8" s="9"/>
       <c r="J8" s="6" t="s">
@@ -1363,13 +1360,13 @@
       </c>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="93"/>
-      <c r="N8" s="77"/>
-      <c r="O8" s="77"/>
+      <c r="M8" s="94"/>
+      <c r="N8" s="95"/>
+      <c r="O8" s="95"/>
       <c r="P8" s="8"/>
     </row>
     <row r="9" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="86" t="s">
+      <c r="B9" s="90" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="79"/>
@@ -1379,7 +1376,7 @@
       <c r="G9" s="79"/>
       <c r="H9" s="80"/>
       <c r="I9" s="9"/>
-      <c r="J9" s="86" t="s">
+      <c r="J9" s="90" t="s">
         <v>3</v>
       </c>
       <c r="K9" s="79"/>
@@ -1411,40 +1408,40 @@
       <c r="P10" s="10"/>
     </row>
     <row r="11" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="96" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="96" t="s">
+      <c r="C11" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="97"/>
-      <c r="E11" s="96" t="s">
+      <c r="D11" s="99"/>
+      <c r="E11" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="97"/>
-      <c r="G11" s="96" t="s">
+      <c r="F11" s="99"/>
+      <c r="G11" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="98"/>
+      <c r="H11" s="100"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="94" t="s">
+      <c r="J11" s="96" t="s">
         <v>5</v>
       </c>
-      <c r="K11" s="96" t="s">
+      <c r="K11" s="98" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="97"/>
-      <c r="M11" s="96" t="s">
+      <c r="L11" s="99"/>
+      <c r="M11" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="N11" s="97"/>
-      <c r="O11" s="96" t="s">
+      <c r="N11" s="99"/>
+      <c r="O11" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="P11" s="98"/>
+      <c r="P11" s="100"/>
     </row>
     <row r="12" spans="2:16" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="95"/>
+      <c r="B12" s="97"/>
       <c r="C12" s="11" t="s">
         <v>9</v>
       </c>
@@ -1464,7 +1461,7 @@
         <v>12</v>
       </c>
       <c r="I12" s="1"/>
-      <c r="J12" s="95"/>
+      <c r="J12" s="97"/>
       <c r="K12" s="74" t="s">
         <v>9</v>
       </c>
@@ -2168,114 +2165,114 @@
       <c r="P44" s="36"/>
     </row>
     <row r="45" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="99"/>
-      <c r="C45" s="100"/>
-      <c r="D45" s="100"/>
-      <c r="E45" s="101"/>
+      <c r="B45" s="81"/>
+      <c r="C45" s="82"/>
+      <c r="D45" s="82"/>
+      <c r="E45" s="83"/>
       <c r="F45" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="G45" s="81"/>
-      <c r="H45" s="82"/>
+      <c r="G45" s="85"/>
+      <c r="H45" s="86"/>
       <c r="I45" s="7"/>
-      <c r="J45" s="99"/>
-      <c r="K45" s="100"/>
-      <c r="L45" s="100"/>
-      <c r="M45" s="101"/>
+      <c r="J45" s="81"/>
+      <c r="K45" s="82"/>
+      <c r="L45" s="82"/>
+      <c r="M45" s="83"/>
       <c r="N45" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="O45" s="81"/>
-      <c r="P45" s="82"/>
+      <c r="O45" s="85"/>
+      <c r="P45" s="86"/>
     </row>
     <row r="46" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="102"/>
+      <c r="B46" s="84"/>
       <c r="C46" s="79"/>
       <c r="D46" s="79"/>
-      <c r="E46" s="101"/>
+      <c r="E46" s="83"/>
       <c r="F46" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="G46" s="81"/>
-      <c r="H46" s="82"/>
+      <c r="G46" s="85"/>
+      <c r="H46" s="86"/>
       <c r="I46" s="7"/>
-      <c r="J46" s="102"/>
+      <c r="J46" s="84"/>
       <c r="K46" s="79"/>
       <c r="L46" s="79"/>
-      <c r="M46" s="101"/>
+      <c r="M46" s="83"/>
       <c r="N46" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="O46" s="81"/>
-      <c r="P46" s="82"/>
+      <c r="O46" s="85"/>
+      <c r="P46" s="86"/>
     </row>
     <row r="47" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="102"/>
+      <c r="B47" s="84"/>
       <c r="C47" s="79"/>
       <c r="D47" s="79"/>
-      <c r="E47" s="101"/>
+      <c r="E47" s="83"/>
       <c r="F47" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="G47" s="81"/>
-      <c r="H47" s="82"/>
+      <c r="G47" s="85"/>
+      <c r="H47" s="86"/>
       <c r="I47" s="7"/>
-      <c r="J47" s="102"/>
+      <c r="J47" s="84"/>
       <c r="K47" s="79"/>
       <c r="L47" s="79"/>
-      <c r="M47" s="101"/>
+      <c r="M47" s="83"/>
       <c r="N47" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="O47" s="81"/>
-      <c r="P47" s="82"/>
+      <c r="O47" s="85"/>
+      <c r="P47" s="86"/>
       <c r="U47" s="29"/>
     </row>
     <row r="48" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="102"/>
+      <c r="B48" s="84"/>
       <c r="C48" s="79"/>
       <c r="D48" s="79"/>
-      <c r="E48" s="101"/>
+      <c r="E48" s="83"/>
       <c r="F48" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="81"/>
-      <c r="H48" s="82"/>
+      <c r="G48" s="85"/>
+      <c r="H48" s="86"/>
       <c r="I48" s="7"/>
-      <c r="J48" s="102"/>
+      <c r="J48" s="84"/>
       <c r="K48" s="79"/>
       <c r="L48" s="79"/>
-      <c r="M48" s="101"/>
+      <c r="M48" s="83"/>
       <c r="N48" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="O48" s="81"/>
-      <c r="P48" s="82"/>
+      <c r="O48" s="85"/>
+      <c r="P48" s="86"/>
       <c r="U48" s="41"/>
     </row>
     <row r="49" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="42"/>
-      <c r="C49" s="83" t="s">
+      <c r="C49" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="84"/>
-      <c r="E49" s="84"/>
-      <c r="F49" s="84"/>
-      <c r="G49" s="84"/>
-      <c r="H49" s="85"/>
+      <c r="D49" s="88"/>
+      <c r="E49" s="88"/>
+      <c r="F49" s="88"/>
+      <c r="G49" s="88"/>
+      <c r="H49" s="89"/>
       <c r="I49" s="7"/>
       <c r="J49" s="42"/>
-      <c r="K49" s="83" t="s">
+      <c r="K49" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="L49" s="84"/>
-      <c r="M49" s="84"/>
-      <c r="N49" s="84"/>
-      <c r="O49" s="84"/>
-      <c r="P49" s="85"/>
+      <c r="L49" s="88"/>
+      <c r="M49" s="88"/>
+      <c r="N49" s="88"/>
+      <c r="O49" s="88"/>
+      <c r="P49" s="89"/>
     </row>
     <row r="50" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="86" t="s">
+      <c r="B50" s="90" t="s">
         <v>19</v>
       </c>
       <c r="C50" s="79"/>
@@ -2285,7 +2282,7 @@
       <c r="G50" s="79"/>
       <c r="H50" s="80"/>
       <c r="I50" s="7"/>
-      <c r="J50" s="86" t="s">
+      <c r="J50" s="90" t="s">
         <v>19</v>
       </c>
       <c r="K50" s="79"/>
@@ -2296,7 +2293,7 @@
       <c r="P50" s="80"/>
     </row>
     <row r="51" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="86" t="s">
+      <c r="B51" s="90" t="s">
         <v>20</v>
       </c>
       <c r="C51" s="79"/>
@@ -2306,7 +2303,7 @@
       <c r="G51" s="79"/>
       <c r="H51" s="80"/>
       <c r="I51" s="9"/>
-      <c r="J51" s="86" t="s">
+      <c r="J51" s="90" t="s">
         <v>20</v>
       </c>
       <c r="K51" s="79"/>
@@ -2317,7 +2314,7 @@
       <c r="P51" s="80"/>
     </row>
     <row r="52" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="86" t="s">
+      <c r="B52" s="90" t="s">
         <v>21</v>
       </c>
       <c r="C52" s="79"/>
@@ -2327,7 +2324,7 @@
       <c r="G52" s="7"/>
       <c r="H52" s="10"/>
       <c r="I52" s="9"/>
-      <c r="J52" s="86" t="s">
+      <c r="J52" s="90" t="s">
         <v>21</v>
       </c>
       <c r="K52" s="79"/>
@@ -2373,23 +2370,23 @@
     </row>
     <row r="55" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="45"/>
-      <c r="C55" s="87"/>
-      <c r="D55" s="88"/>
-      <c r="E55" s="88"/>
-      <c r="F55" s="88"/>
-      <c r="G55" s="88"/>
+      <c r="C55" s="91"/>
+      <c r="D55" s="92"/>
+      <c r="E55" s="92"/>
+      <c r="F55" s="92"/>
+      <c r="G55" s="92"/>
       <c r="H55" s="46"/>
       <c r="I55" s="9"/>
       <c r="J55" s="45"/>
-      <c r="K55" s="87"/>
-      <c r="L55" s="88"/>
-      <c r="M55" s="88"/>
-      <c r="N55" s="88"/>
-      <c r="O55" s="88"/>
+      <c r="K55" s="91"/>
+      <c r="L55" s="92"/>
+      <c r="M55" s="92"/>
+      <c r="N55" s="92"/>
+      <c r="O55" s="92"/>
       <c r="P55" s="46"/>
     </row>
     <row r="56" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="89" t="s">
+      <c r="B56" s="93" t="s">
         <v>22</v>
       </c>
       <c r="C56" s="79"/>
@@ -2399,7 +2396,7 @@
       <c r="G56" s="79"/>
       <c r="H56" s="80"/>
       <c r="I56" s="9"/>
-      <c r="J56" s="89" t="s">
+      <c r="J56" s="93" t="s">
         <v>22</v>
       </c>
       <c r="K56" s="79"/>
@@ -2483,25 +2480,23 @@
     </row>
     <row r="61" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="47"/>
-      <c r="C61" s="76"/>
-      <c r="D61" s="77"/>
-      <c r="E61" s="77"/>
-      <c r="F61" s="77"/>
-      <c r="G61" s="77"/>
+      <c r="C61" s="104"/>
+      <c r="D61" s="95"/>
+      <c r="E61" s="95"/>
+      <c r="F61" s="95"/>
+      <c r="G61" s="95"/>
       <c r="H61" s="48"/>
       <c r="I61" s="9"/>
       <c r="J61" s="47"/>
-      <c r="K61" s="103"/>
-      <c r="L61" s="104"/>
-      <c r="M61" s="104"/>
-      <c r="N61" s="104"/>
-      <c r="O61" s="104"/>
+      <c r="K61" s="76"/>
+      <c r="L61" s="77"/>
+      <c r="M61" s="77"/>
+      <c r="N61" s="77"/>
+      <c r="O61" s="77"/>
       <c r="P61" s="48"/>
     </row>
     <row r="62" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="78" t="s">
-        <v>24</v>
-      </c>
+      <c r="B62" s="78"/>
       <c r="C62" s="79"/>
       <c r="D62" s="79"/>
       <c r="E62" s="79"/>
@@ -2509,9 +2504,7 @@
       <c r="G62" s="79"/>
       <c r="H62" s="80"/>
       <c r="I62" s="49"/>
-      <c r="J62" s="78" t="s">
-        <v>24</v>
-      </c>
+      <c r="J62" s="78"/>
       <c r="K62" s="79"/>
       <c r="L62" s="79"/>
       <c r="M62" s="79"/>
@@ -3482,19 +3475,21 @@
     <row r="1000" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="K61:O61"/>
-    <mergeCell ref="J62:P62"/>
-    <mergeCell ref="J45:M48"/>
-    <mergeCell ref="O45:P45"/>
-    <mergeCell ref="O46:P46"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="O48:P48"/>
-    <mergeCell ref="K49:P49"/>
-    <mergeCell ref="J50:P50"/>
-    <mergeCell ref="J51:P51"/>
-    <mergeCell ref="J52:L52"/>
-    <mergeCell ref="K55:O55"/>
-    <mergeCell ref="J56:P56"/>
+    <mergeCell ref="C61:G61"/>
+    <mergeCell ref="B62:H62"/>
+    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="C49:H49"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="B56:H56"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="J3:P3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="J4:P4"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="K6:O6"/>
     <mergeCell ref="G46:H46"/>
     <mergeCell ref="M8:O8"/>
     <mergeCell ref="J9:P9"/>
@@ -3511,21 +3506,19 @@
     <mergeCell ref="B45:E48"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="G47:H47"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="J3:P3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="J4:P4"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="K6:O6"/>
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="B62:H62"/>
-    <mergeCell ref="G48:H48"/>
-    <mergeCell ref="C49:H49"/>
-    <mergeCell ref="B50:H50"/>
-    <mergeCell ref="B51:H51"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="C55:G55"/>
-    <mergeCell ref="B56:H56"/>
+    <mergeCell ref="K61:O61"/>
+    <mergeCell ref="J62:P62"/>
+    <mergeCell ref="J45:M48"/>
+    <mergeCell ref="O45:P45"/>
+    <mergeCell ref="O46:P46"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="K49:P49"/>
+    <mergeCell ref="J50:P50"/>
+    <mergeCell ref="J51:P51"/>
+    <mergeCell ref="J52:L52"/>
+    <mergeCell ref="K55:O55"/>
+    <mergeCell ref="J56:P56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
updated DTR and AR template files, fixed margin issues
</commit_message>
<xml_diff>
--- a/eaas_python/template_files/DTR_template.xlsx
+++ b/eaas_python/template_files/DTR_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Veronica\Downloads\ver\dict_folder\dict_eeas\eaas_python\template_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B2CA25-67BD-4034-BFA1-4F2EE57B5D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D7C86A-9650-4B8A-B551-E60A0C306DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -106,7 +106,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -175,13 +175,6 @@
     <font>
       <b/>
       <u/>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
@@ -877,10 +870,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -958,21 +951,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -985,17 +972,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1005,18 +996,20 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1252,28 +1245,28 @@
     <row r="1" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="101" t="s">
+      <c r="B3" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="89"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="85"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="101" t="s">
+      <c r="J3" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="88"/>
-      <c r="L3" s="88"/>
-      <c r="M3" s="88"/>
-      <c r="N3" s="88"/>
-      <c r="O3" s="88"/>
-      <c r="P3" s="89"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="84"/>
+      <c r="M3" s="84"/>
+      <c r="N3" s="84"/>
+      <c r="O3" s="84"/>
+      <c r="P3" s="85"/>
     </row>
     <row r="4" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="102" t="s">
+      <c r="B4" s="89" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="79"/>
@@ -1283,7 +1276,7 @@
       <c r="G4" s="79"/>
       <c r="H4" s="80"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="102" t="s">
+      <c r="J4" s="89" t="s">
         <v>1</v>
       </c>
       <c r="K4" s="79"/>
@@ -1312,19 +1305,19 @@
     </row>
     <row r="6" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="95"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="95"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
       <c r="H6" s="5"/>
       <c r="I6" s="1"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="103"/>
-      <c r="L6" s="95"/>
-      <c r="M6" s="95"/>
-      <c r="N6" s="95"/>
-      <c r="O6" s="95"/>
+      <c r="K6" s="90"/>
+      <c r="L6" s="77"/>
+      <c r="M6" s="77"/>
+      <c r="N6" s="77"/>
+      <c r="O6" s="77"/>
       <c r="P6" s="5"/>
     </row>
     <row r="7" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1350,9 +1343,9 @@
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="94"/>
-      <c r="F8" s="95"/>
-      <c r="G8" s="95"/>
+      <c r="E8" s="91"/>
+      <c r="F8" s="77"/>
+      <c r="G8" s="77"/>
       <c r="H8" s="8"/>
       <c r="I8" s="9"/>
       <c r="J8" s="6" t="s">
@@ -1360,13 +1353,13 @@
       </c>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="94"/>
-      <c r="N8" s="95"/>
-      <c r="O8" s="95"/>
+      <c r="M8" s="91"/>
+      <c r="N8" s="77"/>
+      <c r="O8" s="77"/>
       <c r="P8" s="8"/>
     </row>
     <row r="9" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="90" t="s">
+      <c r="B9" s="86" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="79"/>
@@ -1376,7 +1369,7 @@
       <c r="G9" s="79"/>
       <c r="H9" s="80"/>
       <c r="I9" s="9"/>
-      <c r="J9" s="90" t="s">
+      <c r="J9" s="86" t="s">
         <v>3</v>
       </c>
       <c r="K9" s="79"/>
@@ -1408,40 +1401,40 @@
       <c r="P10" s="10"/>
     </row>
     <row r="11" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="96" t="s">
+      <c r="B11" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="98" t="s">
+      <c r="C11" s="94" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="99"/>
-      <c r="E11" s="98" t="s">
+      <c r="D11" s="95"/>
+      <c r="E11" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="99"/>
-      <c r="G11" s="98" t="s">
+      <c r="F11" s="95"/>
+      <c r="G11" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="100"/>
+      <c r="H11" s="96"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="96" t="s">
+      <c r="J11" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="K11" s="98" t="s">
+      <c r="K11" s="94" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="99"/>
-      <c r="M11" s="98" t="s">
+      <c r="L11" s="95"/>
+      <c r="M11" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="N11" s="99"/>
-      <c r="O11" s="98" t="s">
+      <c r="N11" s="95"/>
+      <c r="O11" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="P11" s="100"/>
+      <c r="P11" s="96"/>
     </row>
     <row r="12" spans="2:16" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="97"/>
+      <c r="B12" s="93"/>
       <c r="C12" s="11" t="s">
         <v>9</v>
       </c>
@@ -1461,7 +1454,7 @@
         <v>12</v>
       </c>
       <c r="I12" s="1"/>
-      <c r="J12" s="97"/>
+      <c r="J12" s="93"/>
       <c r="K12" s="74" t="s">
         <v>9</v>
       </c>
@@ -2165,114 +2158,114 @@
       <c r="P44" s="36"/>
     </row>
     <row r="45" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="81"/>
-      <c r="C45" s="82"/>
-      <c r="D45" s="82"/>
-      <c r="E45" s="83"/>
+      <c r="B45" s="97"/>
+      <c r="C45" s="98"/>
+      <c r="D45" s="98"/>
+      <c r="E45" s="99"/>
       <c r="F45" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="G45" s="85"/>
-      <c r="H45" s="86"/>
+      <c r="G45" s="81"/>
+      <c r="H45" s="82"/>
       <c r="I45" s="7"/>
-      <c r="J45" s="81"/>
-      <c r="K45" s="82"/>
-      <c r="L45" s="82"/>
-      <c r="M45" s="83"/>
+      <c r="J45" s="97"/>
+      <c r="K45" s="98"/>
+      <c r="L45" s="98"/>
+      <c r="M45" s="99"/>
       <c r="N45" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="O45" s="85"/>
-      <c r="P45" s="86"/>
+      <c r="O45" s="81"/>
+      <c r="P45" s="82"/>
     </row>
     <row r="46" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="84"/>
+      <c r="B46" s="100"/>
       <c r="C46" s="79"/>
       <c r="D46" s="79"/>
-      <c r="E46" s="83"/>
+      <c r="E46" s="99"/>
       <c r="F46" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="G46" s="85"/>
-      <c r="H46" s="86"/>
+      <c r="G46" s="81"/>
+      <c r="H46" s="82"/>
       <c r="I46" s="7"/>
-      <c r="J46" s="84"/>
+      <c r="J46" s="100"/>
       <c r="K46" s="79"/>
       <c r="L46" s="79"/>
-      <c r="M46" s="83"/>
+      <c r="M46" s="99"/>
       <c r="N46" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="O46" s="85"/>
-      <c r="P46" s="86"/>
+      <c r="O46" s="81"/>
+      <c r="P46" s="82"/>
     </row>
     <row r="47" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="84"/>
+      <c r="B47" s="100"/>
       <c r="C47" s="79"/>
       <c r="D47" s="79"/>
-      <c r="E47" s="83"/>
+      <c r="E47" s="99"/>
       <c r="F47" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="G47" s="85"/>
-      <c r="H47" s="86"/>
+      <c r="G47" s="81"/>
+      <c r="H47" s="82"/>
       <c r="I47" s="7"/>
-      <c r="J47" s="84"/>
+      <c r="J47" s="100"/>
       <c r="K47" s="79"/>
       <c r="L47" s="79"/>
-      <c r="M47" s="83"/>
+      <c r="M47" s="99"/>
       <c r="N47" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="O47" s="85"/>
-      <c r="P47" s="86"/>
+      <c r="O47" s="81"/>
+      <c r="P47" s="82"/>
       <c r="U47" s="29"/>
     </row>
     <row r="48" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="84"/>
+      <c r="B48" s="100"/>
       <c r="C48" s="79"/>
       <c r="D48" s="79"/>
-      <c r="E48" s="83"/>
+      <c r="E48" s="99"/>
       <c r="F48" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="85"/>
-      <c r="H48" s="86"/>
+      <c r="G48" s="81"/>
+      <c r="H48" s="82"/>
       <c r="I48" s="7"/>
-      <c r="J48" s="84"/>
+      <c r="J48" s="100"/>
       <c r="K48" s="79"/>
       <c r="L48" s="79"/>
-      <c r="M48" s="83"/>
+      <c r="M48" s="99"/>
       <c r="N48" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="O48" s="85"/>
-      <c r="P48" s="86"/>
+      <c r="O48" s="81"/>
+      <c r="P48" s="82"/>
       <c r="U48" s="41"/>
     </row>
     <row r="49" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="42"/>
-      <c r="C49" s="87" t="s">
+      <c r="C49" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="88"/>
-      <c r="E49" s="88"/>
-      <c r="F49" s="88"/>
-      <c r="G49" s="88"/>
-      <c r="H49" s="89"/>
+      <c r="D49" s="84"/>
+      <c r="E49" s="84"/>
+      <c r="F49" s="84"/>
+      <c r="G49" s="84"/>
+      <c r="H49" s="85"/>
       <c r="I49" s="7"/>
       <c r="J49" s="42"/>
-      <c r="K49" s="87" t="s">
+      <c r="K49" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="L49" s="88"/>
-      <c r="M49" s="88"/>
-      <c r="N49" s="88"/>
-      <c r="O49" s="88"/>
-      <c r="P49" s="89"/>
+      <c r="L49" s="84"/>
+      <c r="M49" s="84"/>
+      <c r="N49" s="84"/>
+      <c r="O49" s="84"/>
+      <c r="P49" s="85"/>
     </row>
     <row r="50" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="90" t="s">
+      <c r="B50" s="86" t="s">
         <v>19</v>
       </c>
       <c r="C50" s="79"/>
@@ -2282,7 +2275,7 @@
       <c r="G50" s="79"/>
       <c r="H50" s="80"/>
       <c r="I50" s="7"/>
-      <c r="J50" s="90" t="s">
+      <c r="J50" s="86" t="s">
         <v>19</v>
       </c>
       <c r="K50" s="79"/>
@@ -2293,7 +2286,7 @@
       <c r="P50" s="80"/>
     </row>
     <row r="51" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="90" t="s">
+      <c r="B51" s="86" t="s">
         <v>20</v>
       </c>
       <c r="C51" s="79"/>
@@ -2303,7 +2296,7 @@
       <c r="G51" s="79"/>
       <c r="H51" s="80"/>
       <c r="I51" s="9"/>
-      <c r="J51" s="90" t="s">
+      <c r="J51" s="86" t="s">
         <v>20</v>
       </c>
       <c r="K51" s="79"/>
@@ -2314,7 +2307,7 @@
       <c r="P51" s="80"/>
     </row>
     <row r="52" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="90" t="s">
+      <c r="B52" s="86" t="s">
         <v>21</v>
       </c>
       <c r="C52" s="79"/>
@@ -2324,7 +2317,7 @@
       <c r="G52" s="7"/>
       <c r="H52" s="10"/>
       <c r="I52" s="9"/>
-      <c r="J52" s="90" t="s">
+      <c r="J52" s="86" t="s">
         <v>21</v>
       </c>
       <c r="K52" s="79"/>
@@ -2370,23 +2363,23 @@
     </row>
     <row r="55" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="45"/>
-      <c r="C55" s="91"/>
-      <c r="D55" s="92"/>
-      <c r="E55" s="92"/>
-      <c r="F55" s="92"/>
-      <c r="G55" s="92"/>
+      <c r="C55" s="103"/>
+      <c r="D55" s="104"/>
+      <c r="E55" s="104"/>
+      <c r="F55" s="104"/>
+      <c r="G55" s="104"/>
       <c r="H55" s="46"/>
       <c r="I55" s="9"/>
       <c r="J55" s="45"/>
-      <c r="K55" s="91"/>
-      <c r="L55" s="92"/>
-      <c r="M55" s="92"/>
-      <c r="N55" s="92"/>
-      <c r="O55" s="92"/>
+      <c r="K55" s="103"/>
+      <c r="L55" s="104"/>
+      <c r="M55" s="104"/>
+      <c r="N55" s="104"/>
+      <c r="O55" s="104"/>
       <c r="P55" s="46"/>
     </row>
     <row r="56" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="93" t="s">
+      <c r="B56" s="87" t="s">
         <v>22</v>
       </c>
       <c r="C56" s="79"/>
@@ -2396,7 +2389,7 @@
       <c r="G56" s="79"/>
       <c r="H56" s="80"/>
       <c r="I56" s="9"/>
-      <c r="J56" s="93" t="s">
+      <c r="J56" s="87" t="s">
         <v>22</v>
       </c>
       <c r="K56" s="79"/>
@@ -2480,19 +2473,19 @@
     </row>
     <row r="61" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="47"/>
-      <c r="C61" s="104"/>
-      <c r="D61" s="95"/>
-      <c r="E61" s="95"/>
-      <c r="F61" s="95"/>
-      <c r="G61" s="95"/>
+      <c r="C61" s="76"/>
+      <c r="D61" s="77"/>
+      <c r="E61" s="77"/>
+      <c r="F61" s="77"/>
+      <c r="G61" s="77"/>
       <c r="H61" s="48"/>
       <c r="I61" s="9"/>
       <c r="J61" s="47"/>
-      <c r="K61" s="76"/>
-      <c r="L61" s="77"/>
-      <c r="M61" s="77"/>
-      <c r="N61" s="77"/>
-      <c r="O61" s="77"/>
+      <c r="K61" s="101"/>
+      <c r="L61" s="102"/>
+      <c r="M61" s="102"/>
+      <c r="N61" s="102"/>
+      <c r="O61" s="102"/>
       <c r="P61" s="48"/>
     </row>
     <row r="62" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3475,21 +3468,19 @@
     <row r="1000" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="B62:H62"/>
-    <mergeCell ref="G48:H48"/>
-    <mergeCell ref="C49:H49"/>
-    <mergeCell ref="B50:H50"/>
-    <mergeCell ref="B51:H51"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="C55:G55"/>
-    <mergeCell ref="B56:H56"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="J3:P3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="J4:P4"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="K6:O6"/>
+    <mergeCell ref="K61:O61"/>
+    <mergeCell ref="J62:P62"/>
+    <mergeCell ref="J45:M48"/>
+    <mergeCell ref="O45:P45"/>
+    <mergeCell ref="O46:P46"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="K49:P49"/>
+    <mergeCell ref="J50:P50"/>
+    <mergeCell ref="J51:P51"/>
+    <mergeCell ref="J52:L52"/>
+    <mergeCell ref="K55:O55"/>
+    <mergeCell ref="J56:P56"/>
     <mergeCell ref="G46:H46"/>
     <mergeCell ref="M8:O8"/>
     <mergeCell ref="J9:P9"/>
@@ -3506,19 +3497,21 @@
     <mergeCell ref="B45:E48"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="G47:H47"/>
-    <mergeCell ref="K61:O61"/>
-    <mergeCell ref="J62:P62"/>
-    <mergeCell ref="J45:M48"/>
-    <mergeCell ref="O45:P45"/>
-    <mergeCell ref="O46:P46"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="O48:P48"/>
-    <mergeCell ref="K49:P49"/>
-    <mergeCell ref="J50:P50"/>
-    <mergeCell ref="J51:P51"/>
-    <mergeCell ref="J52:L52"/>
-    <mergeCell ref="K55:O55"/>
-    <mergeCell ref="J56:P56"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="J3:P3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="J4:P4"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="K6:O6"/>
+    <mergeCell ref="C61:G61"/>
+    <mergeCell ref="B62:H62"/>
+    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="C49:H49"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="B56:H56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
>No Claim/With Claim remarks >DTR now has 2 templates >Office hours are now a thing, set by admin, affects undertime computation >Undertime is now computed automatically, based on time entries, office hours, and whatever the employee types into the time entries >cells in a row can now be merge manually
</commit_message>
<xml_diff>
--- a/eaas_python/template_files/DTR_template.xlsx
+++ b/eaas_python/template_files/DTR_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Veronica\Downloads\ver\dict_folder\dict_eeas\eaas_python\template_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D7C86A-9650-4B8A-B551-E60A0C306DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE88AED-22F3-454E-9B47-9C5AE4F7C425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -106,7 +106,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -117,26 +117,31 @@
       <sz val="8"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -144,33 +149,33 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF333333"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -178,12 +183,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -191,6 +198,57 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -734,7 +792,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -772,87 +830,27 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="20" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -870,10 +868,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -889,69 +887,46 @@
     <xf numFmtId="164" fontId="8" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="5" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -972,6 +947,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1002,14 +981,103 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="14" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="14" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1228,7 +1296,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:X1000"/>
+  <dimension ref="A1:X1000"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.44140625" customWidth="1"/>
@@ -1242,51 +1310,51 @@
     <col min="17" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="88" t="s">
+    <row r="1" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="84"/>
-      <c r="H3" s="85"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="56"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="88" t="s">
+      <c r="J3" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="84"/>
-      <c r="L3" s="84"/>
-      <c r="M3" s="84"/>
-      <c r="N3" s="84"/>
-      <c r="O3" s="84"/>
-      <c r="P3" s="85"/>
-    </row>
-    <row r="4" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="89" t="s">
+      <c r="K3" s="55"/>
+      <c r="L3" s="55"/>
+      <c r="M3" s="55"/>
+      <c r="N3" s="55"/>
+      <c r="O3" s="55"/>
+      <c r="P3" s="56"/>
+    </row>
+    <row r="4" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="80"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="51"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="89" t="s">
+      <c r="J4" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-      <c r="N4" s="79"/>
-      <c r="O4" s="79"/>
-      <c r="P4" s="80"/>
-    </row>
-    <row r="5" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K4" s="50"/>
+      <c r="L4" s="50"/>
+      <c r="M4" s="50"/>
+      <c r="N4" s="50"/>
+      <c r="O4" s="50"/>
+      <c r="P4" s="51"/>
+    </row>
+    <row r="5" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1303,24 +1371,24 @@
       <c r="O5" s="1"/>
       <c r="P5" s="4"/>
     </row>
-    <row r="6" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
-      <c r="C6" s="90"/>
-      <c r="D6" s="77"/>
-      <c r="E6" s="77"/>
-      <c r="F6" s="77"/>
-      <c r="G6" s="77"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
       <c r="H6" s="5"/>
       <c r="I6" s="1"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="90"/>
-      <c r="L6" s="77"/>
-      <c r="M6" s="77"/>
-      <c r="N6" s="77"/>
-      <c r="O6" s="77"/>
+      <c r="K6" s="63"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
       <c r="P6" s="5"/>
     </row>
-    <row r="7" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1337,15 +1405,15 @@
       <c r="O7" s="1"/>
       <c r="P7" s="4"/>
     </row>
-    <row r="8" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="77"/>
-      <c r="G8" s="77"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
       <c r="H8" s="8"/>
       <c r="I8" s="9"/>
       <c r="J8" s="6" t="s">
@@ -1353,33 +1421,33 @@
       </c>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="91"/>
-      <c r="N8" s="77"/>
-      <c r="O8" s="77"/>
+      <c r="M8" s="64"/>
+      <c r="N8" s="48"/>
+      <c r="O8" s="48"/>
       <c r="P8" s="8"/>
     </row>
-    <row r="9" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="86" t="s">
+    <row r="9" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="79"/>
-      <c r="D9" s="79"/>
-      <c r="E9" s="79"/>
-      <c r="F9" s="79"/>
-      <c r="G9" s="79"/>
-      <c r="H9" s="80"/>
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="51"/>
       <c r="I9" s="9"/>
-      <c r="J9" s="86" t="s">
+      <c r="J9" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="K9" s="79"/>
-      <c r="L9" s="79"/>
-      <c r="M9" s="79"/>
-      <c r="N9" s="79"/>
-      <c r="O9" s="79"/>
-      <c r="P9" s="80"/>
-    </row>
-    <row r="10" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="50"/>
+      <c r="O9" s="50"/>
+      <c r="P9" s="51"/>
+    </row>
+    <row r="10" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
@@ -1400,41 +1468,41 @@
       <c r="O10" s="7"/>
       <c r="P10" s="10"/>
     </row>
-    <row r="11" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="92" t="s">
+    <row r="11" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="94" t="s">
+      <c r="C11" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="95"/>
-      <c r="E11" s="94" t="s">
+      <c r="D11" s="68"/>
+      <c r="E11" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="95"/>
-      <c r="G11" s="94" t="s">
+      <c r="F11" s="68"/>
+      <c r="G11" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="96"/>
+      <c r="H11" s="69"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="92" t="s">
+      <c r="J11" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="K11" s="94" t="s">
+      <c r="K11" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="95"/>
-      <c r="M11" s="94" t="s">
+      <c r="L11" s="68"/>
+      <c r="M11" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="N11" s="95"/>
-      <c r="O11" s="94" t="s">
+      <c r="N11" s="68"/>
+      <c r="O11" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="P11" s="96"/>
-    </row>
-    <row r="12" spans="2:16" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="93"/>
+      <c r="P11" s="69"/>
+    </row>
+    <row r="12" spans="1:17" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="66"/>
       <c r="C12" s="11" t="s">
         <v>9</v>
       </c>
@@ -1454,17 +1522,17 @@
         <v>12</v>
       </c>
       <c r="I12" s="1"/>
-      <c r="J12" s="93"/>
-      <c r="K12" s="74" t="s">
+      <c r="J12" s="66"/>
+      <c r="K12" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="L12" s="75" t="s">
+      <c r="L12" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="M12" s="75" t="s">
+      <c r="M12" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="N12" s="75" t="s">
+      <c r="N12" s="46" t="s">
         <v>10</v>
       </c>
       <c r="O12" s="11" t="s">
@@ -1474,933 +1542,997 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="13"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="73"/>
-      <c r="L13" s="73"/>
-      <c r="M13" s="73"/>
-      <c r="N13" s="73"/>
-      <c r="O13" s="72"/>
-      <c r="P13" s="16"/>
-    </row>
-    <row r="14" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="17">
+    <row r="13" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="108"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="78"/>
+      <c r="H13" s="79"/>
+      <c r="I13" s="80"/>
+      <c r="J13" s="76"/>
+      <c r="K13" s="81"/>
+      <c r="L13" s="81"/>
+      <c r="M13" s="81"/>
+      <c r="N13" s="81"/>
+      <c r="O13" s="82"/>
+      <c r="P13" s="79"/>
+      <c r="Q13" s="108"/>
+    </row>
+    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="108"/>
+      <c r="B14" s="83">
         <v>1</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="17">
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="84"/>
+      <c r="H14" s="85"/>
+      <c r="I14" s="86"/>
+      <c r="J14" s="83">
         <v>1</v>
       </c>
-      <c r="K14" s="69"/>
-      <c r="L14" s="69"/>
-      <c r="M14" s="69"/>
-      <c r="N14" s="69"/>
-      <c r="O14" s="54"/>
-      <c r="P14" s="20"/>
-    </row>
-    <row r="15" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="22">
+      <c r="K14" s="43"/>
+      <c r="L14" s="43"/>
+      <c r="M14" s="43"/>
+      <c r="N14" s="43"/>
+      <c r="O14" s="87"/>
+      <c r="P14" s="85"/>
+      <c r="Q14" s="108"/>
+    </row>
+    <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="108"/>
+      <c r="B15" s="88">
         <v>2</v>
       </c>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="22">
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="84"/>
+      <c r="H15" s="85"/>
+      <c r="I15" s="86"/>
+      <c r="J15" s="88">
         <v>2</v>
       </c>
-      <c r="K15" s="69"/>
-      <c r="L15" s="69"/>
-      <c r="M15" s="69"/>
-      <c r="N15" s="69"/>
-      <c r="O15" s="54"/>
-      <c r="P15" s="20"/>
-    </row>
-    <row r="16" spans="2:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="22">
+      <c r="K15" s="43"/>
+      <c r="L15" s="43"/>
+      <c r="M15" s="43"/>
+      <c r="N15" s="43"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="85"/>
+      <c r="Q15" s="108"/>
+    </row>
+    <row r="16" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="108"/>
+      <c r="B16" s="88">
         <v>3</v>
       </c>
-      <c r="C16" s="64"/>
-      <c r="D16" s="65"/>
-      <c r="E16" s="65"/>
-      <c r="F16" s="65"/>
-      <c r="G16" s="54"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="22">
+      <c r="C16" s="39"/>
+      <c r="D16" s="89"/>
+      <c r="E16" s="89"/>
+      <c r="F16" s="89"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="85"/>
+      <c r="I16" s="86"/>
+      <c r="J16" s="88">
         <v>3</v>
       </c>
-      <c r="K16" s="64"/>
-      <c r="L16" s="65"/>
-      <c r="M16" s="65"/>
-      <c r="N16" s="65"/>
-      <c r="O16" s="54"/>
-      <c r="P16" s="20"/>
-    </row>
-    <row r="17" spans="2:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="22">
+      <c r="K16" s="39"/>
+      <c r="L16" s="89"/>
+      <c r="M16" s="89"/>
+      <c r="N16" s="89"/>
+      <c r="O16" s="87"/>
+      <c r="P16" s="85"/>
+      <c r="Q16" s="108"/>
+    </row>
+    <row r="17" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="108"/>
+      <c r="B17" s="88">
         <v>4</v>
       </c>
-      <c r="C17" s="64"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="65"/>
-      <c r="F17" s="65"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="22">
+      <c r="C17" s="39"/>
+      <c r="D17" s="89"/>
+      <c r="E17" s="89"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="90"/>
+      <c r="H17" s="91"/>
+      <c r="I17" s="86"/>
+      <c r="J17" s="88">
         <v>4</v>
       </c>
-      <c r="K17" s="64"/>
-      <c r="L17" s="65"/>
-      <c r="M17" s="65"/>
-      <c r="N17" s="65"/>
-      <c r="O17" s="55"/>
-      <c r="P17" s="23"/>
-    </row>
-    <row r="18" spans="2:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="22">
+      <c r="K17" s="39"/>
+      <c r="L17" s="89"/>
+      <c r="M17" s="89"/>
+      <c r="N17" s="89"/>
+      <c r="O17" s="90"/>
+      <c r="P17" s="91"/>
+      <c r="Q17" s="108"/>
+    </row>
+    <row r="18" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="108"/>
+      <c r="B18" s="88">
         <v>5</v>
       </c>
-      <c r="C18" s="64"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="65"/>
-      <c r="F18" s="65"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="22">
+      <c r="C18" s="39"/>
+      <c r="D18" s="89"/>
+      <c r="E18" s="89"/>
+      <c r="F18" s="89"/>
+      <c r="G18" s="90"/>
+      <c r="H18" s="85"/>
+      <c r="I18" s="86"/>
+      <c r="J18" s="88">
         <v>5</v>
       </c>
-      <c r="K18" s="64"/>
-      <c r="L18" s="65"/>
-      <c r="M18" s="65"/>
-      <c r="N18" s="65"/>
-      <c r="O18" s="55"/>
-      <c r="P18" s="20"/>
-    </row>
-    <row r="19" spans="2:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="22">
+      <c r="K18" s="39"/>
+      <c r="L18" s="89"/>
+      <c r="M18" s="89"/>
+      <c r="N18" s="89"/>
+      <c r="O18" s="90"/>
+      <c r="P18" s="85"/>
+      <c r="Q18" s="108"/>
+    </row>
+    <row r="19" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="108"/>
+      <c r="B19" s="88">
         <v>6</v>
       </c>
-      <c r="C19" s="61"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="22">
+      <c r="C19" s="36"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="92"/>
+      <c r="H19" s="93"/>
+      <c r="I19" s="94"/>
+      <c r="J19" s="88">
         <v>6</v>
       </c>
-      <c r="K19" s="69"/>
-      <c r="L19" s="69"/>
-      <c r="M19" s="69"/>
-      <c r="N19" s="69"/>
-      <c r="O19" s="56"/>
-      <c r="P19" s="24"/>
-      <c r="X19" s="25"/>
-    </row>
-    <row r="20" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="22">
+      <c r="K19" s="43"/>
+      <c r="L19" s="43"/>
+      <c r="M19" s="43"/>
+      <c r="N19" s="43"/>
+      <c r="O19" s="92"/>
+      <c r="P19" s="93"/>
+      <c r="Q19" s="108"/>
+      <c r="X19" s="14"/>
+    </row>
+    <row r="20" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="108"/>
+      <c r="B20" s="88">
         <v>7</v>
       </c>
-      <c r="C20" s="53"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="59"/>
-      <c r="G20" s="54"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="22">
+      <c r="C20" s="33"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="87"/>
+      <c r="H20" s="85"/>
+      <c r="I20" s="80"/>
+      <c r="J20" s="88">
         <v>7</v>
       </c>
-      <c r="K20" s="69"/>
-      <c r="L20" s="69"/>
-      <c r="M20" s="69"/>
-      <c r="N20" s="69"/>
-      <c r="O20" s="54"/>
-      <c r="P20" s="20"/>
-    </row>
-    <row r="21" spans="2:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="22">
+      <c r="K20" s="43"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="43"/>
+      <c r="N20" s="43"/>
+      <c r="O20" s="87"/>
+      <c r="P20" s="85"/>
+      <c r="Q20" s="108"/>
+    </row>
+    <row r="21" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="108"/>
+      <c r="B21" s="88">
         <v>8</v>
       </c>
-      <c r="C21" s="53"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="22">
+      <c r="C21" s="33"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="91"/>
+      <c r="I21" s="80"/>
+      <c r="J21" s="88">
         <v>8</v>
       </c>
-      <c r="K21" s="69"/>
-      <c r="L21" s="69"/>
-      <c r="M21" s="69"/>
-      <c r="N21" s="69"/>
-      <c r="O21" s="54"/>
-      <c r="P21" s="23"/>
-    </row>
-    <row r="22" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="22">
+      <c r="K21" s="43"/>
+      <c r="L21" s="43"/>
+      <c r="M21" s="43"/>
+      <c r="N21" s="43"/>
+      <c r="O21" s="87"/>
+      <c r="P21" s="91"/>
+      <c r="Q21" s="108"/>
+    </row>
+    <row r="22" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="108"/>
+      <c r="B22" s="88">
         <v>9</v>
       </c>
-      <c r="C22" s="66"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="67"/>
-      <c r="G22" s="54"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="22">
+      <c r="C22" s="40"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="85"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="88">
         <v>9</v>
       </c>
-      <c r="K22" s="69"/>
-      <c r="L22" s="69"/>
-      <c r="M22" s="69"/>
-      <c r="N22" s="69"/>
-      <c r="O22" s="54"/>
-      <c r="P22" s="20"/>
-    </row>
-    <row r="23" spans="2:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="22">
+      <c r="K22" s="43"/>
+      <c r="L22" s="43"/>
+      <c r="M22" s="43"/>
+      <c r="N22" s="43"/>
+      <c r="O22" s="87"/>
+      <c r="P22" s="85"/>
+      <c r="Q22" s="108"/>
+    </row>
+    <row r="23" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="108"/>
+      <c r="B23" s="88">
         <v>10</v>
       </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="65"/>
-      <c r="E23" s="65"/>
-      <c r="F23" s="65"/>
-      <c r="G23" s="55"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="22">
+      <c r="C23" s="44"/>
+      <c r="D23" s="89"/>
+      <c r="E23" s="89"/>
+      <c r="F23" s="89"/>
+      <c r="G23" s="90"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="80"/>
+      <c r="J23" s="88">
         <v>10</v>
       </c>
-      <c r="K23" s="64"/>
-      <c r="L23" s="65"/>
-      <c r="M23" s="65"/>
-      <c r="N23" s="65"/>
-      <c r="O23" s="55"/>
-      <c r="P23" s="20"/>
-    </row>
-    <row r="24" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="22">
+      <c r="K23" s="39"/>
+      <c r="L23" s="89"/>
+      <c r="M23" s="89"/>
+      <c r="N23" s="89"/>
+      <c r="O23" s="90"/>
+      <c r="P23" s="85"/>
+      <c r="Q23" s="108"/>
+    </row>
+    <row r="24" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="108"/>
+      <c r="B24" s="88">
         <v>11</v>
       </c>
-      <c r="C24" s="71"/>
-      <c r="D24" s="65"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="65"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="22">
+      <c r="C24" s="44"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="89"/>
+      <c r="F24" s="89"/>
+      <c r="G24" s="90"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="80"/>
+      <c r="J24" s="88">
         <v>11</v>
       </c>
-      <c r="K24" s="64"/>
-      <c r="L24" s="65"/>
-      <c r="M24" s="65"/>
-      <c r="N24" s="65"/>
-      <c r="O24" s="55"/>
-      <c r="P24" s="20"/>
-    </row>
-    <row r="25" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="22">
+      <c r="K24" s="39"/>
+      <c r="L24" s="89"/>
+      <c r="M24" s="89"/>
+      <c r="N24" s="89"/>
+      <c r="O24" s="90"/>
+      <c r="P24" s="85"/>
+      <c r="Q24" s="108"/>
+    </row>
+    <row r="25" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="108"/>
+      <c r="B25" s="88">
         <v>12</v>
       </c>
-      <c r="C25" s="71"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="65"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="22">
+      <c r="C25" s="44"/>
+      <c r="D25" s="89"/>
+      <c r="E25" s="89"/>
+      <c r="F25" s="89"/>
+      <c r="G25" s="95"/>
+      <c r="H25" s="96"/>
+      <c r="I25" s="97"/>
+      <c r="J25" s="88">
         <v>12</v>
       </c>
-      <c r="K25" s="64"/>
-      <c r="L25" s="65"/>
-      <c r="M25" s="65"/>
-      <c r="N25" s="65"/>
-      <c r="O25" s="57"/>
-      <c r="P25" s="26"/>
-      <c r="U25" s="28"/>
-      <c r="V25" s="29"/>
-      <c r="W25" s="28"/>
-    </row>
-    <row r="26" spans="2:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="22">
+      <c r="K25" s="39"/>
+      <c r="L25" s="89"/>
+      <c r="M25" s="89"/>
+      <c r="N25" s="89"/>
+      <c r="O25" s="95"/>
+      <c r="P25" s="96"/>
+      <c r="Q25" s="108"/>
+      <c r="U25" s="15"/>
+      <c r="V25" s="16"/>
+      <c r="W25" s="15"/>
+    </row>
+    <row r="26" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="108"/>
+      <c r="B26" s="88">
         <v>13</v>
       </c>
-      <c r="C26" s="69"/>
-      <c r="D26" s="69"/>
-      <c r="E26" s="69"/>
-      <c r="F26" s="69"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="22">
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="98"/>
+      <c r="H26" s="99"/>
+      <c r="I26" s="97"/>
+      <c r="J26" s="88">
         <v>13</v>
       </c>
-      <c r="K26" s="69"/>
-      <c r="L26" s="69"/>
-      <c r="M26" s="69"/>
-      <c r="N26" s="69"/>
-      <c r="O26" s="58"/>
-      <c r="P26" s="30"/>
-      <c r="U26" s="28"/>
-      <c r="V26" s="29"/>
-      <c r="W26" s="28"/>
-    </row>
-    <row r="27" spans="2:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="22">
+      <c r="K26" s="43"/>
+      <c r="L26" s="43"/>
+      <c r="M26" s="43"/>
+      <c r="N26" s="43"/>
+      <c r="O26" s="98"/>
+      <c r="P26" s="99"/>
+      <c r="Q26" s="108"/>
+      <c r="U26" s="15"/>
+      <c r="V26" s="16"/>
+      <c r="W26" s="15"/>
+    </row>
+    <row r="27" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="108"/>
+      <c r="B27" s="88">
         <v>14</v>
       </c>
-      <c r="C27" s="69"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="69"/>
-      <c r="G27" s="58"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="22">
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="98"/>
+      <c r="H27" s="99"/>
+      <c r="I27" s="100"/>
+      <c r="J27" s="88">
         <v>14</v>
       </c>
-      <c r="K27" s="69"/>
-      <c r="L27" s="69"/>
-      <c r="M27" s="69"/>
-      <c r="N27" s="69"/>
-      <c r="O27" s="58"/>
-      <c r="P27" s="30"/>
-      <c r="W27" s="25"/>
-    </row>
-    <row r="28" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="22">
+      <c r="K27" s="43"/>
+      <c r="L27" s="43"/>
+      <c r="M27" s="43"/>
+      <c r="N27" s="43"/>
+      <c r="O27" s="98"/>
+      <c r="P27" s="99"/>
+      <c r="Q27" s="108"/>
+      <c r="W27" s="14"/>
+    </row>
+    <row r="28" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="108"/>
+      <c r="B28" s="88">
         <v>15</v>
       </c>
-      <c r="C28" s="69"/>
-      <c r="D28" s="69"/>
-      <c r="E28" s="69"/>
-      <c r="F28" s="69"/>
-      <c r="G28" s="57"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="22">
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="95"/>
+      <c r="H28" s="101"/>
+      <c r="I28" s="100"/>
+      <c r="J28" s="88">
         <v>15</v>
       </c>
-      <c r="K28" s="69"/>
-      <c r="L28" s="69"/>
-      <c r="M28" s="69"/>
-      <c r="N28" s="69"/>
-      <c r="O28" s="57"/>
-      <c r="P28" s="32"/>
-    </row>
-    <row r="29" spans="2:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="22">
+      <c r="K28" s="43"/>
+      <c r="L28" s="43"/>
+      <c r="M28" s="43"/>
+      <c r="N28" s="43"/>
+      <c r="O28" s="95"/>
+      <c r="P28" s="101"/>
+      <c r="Q28" s="108"/>
+    </row>
+    <row r="29" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="108"/>
+      <c r="B29" s="88">
         <v>16</v>
       </c>
-      <c r="C29" s="69"/>
-      <c r="D29" s="69"/>
-      <c r="E29" s="69"/>
-      <c r="F29" s="69"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="22">
+      <c r="C29" s="43"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="92"/>
+      <c r="H29" s="102"/>
+      <c r="I29" s="80"/>
+      <c r="J29" s="88">
         <v>16</v>
       </c>
-      <c r="K29" s="69"/>
-      <c r="L29" s="69"/>
-      <c r="M29" s="69"/>
-      <c r="N29" s="69"/>
-      <c r="O29" s="56"/>
-      <c r="P29" s="33"/>
-    </row>
-    <row r="30" spans="2:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="22">
+      <c r="K29" s="43"/>
+      <c r="L29" s="43"/>
+      <c r="M29" s="43"/>
+      <c r="N29" s="43"/>
+      <c r="O29" s="92"/>
+      <c r="P29" s="102"/>
+      <c r="Q29" s="108"/>
+    </row>
+    <row r="30" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="108"/>
+      <c r="B30" s="88">
         <v>17</v>
       </c>
-      <c r="C30" s="69"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="22">
+      <c r="C30" s="43"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="90"/>
+      <c r="H30" s="103"/>
+      <c r="I30" s="80"/>
+      <c r="J30" s="88">
         <v>17</v>
       </c>
-      <c r="K30" s="69"/>
-      <c r="L30" s="69"/>
-      <c r="M30" s="69"/>
-      <c r="N30" s="69"/>
-      <c r="O30" s="55"/>
-      <c r="P30" s="34"/>
-    </row>
-    <row r="31" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="22">
+      <c r="K30" s="43"/>
+      <c r="L30" s="43"/>
+      <c r="M30" s="43"/>
+      <c r="N30" s="43"/>
+      <c r="O30" s="90"/>
+      <c r="P30" s="103"/>
+      <c r="Q30" s="108"/>
+    </row>
+    <row r="31" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="108"/>
+      <c r="B31" s="88">
         <v>18</v>
       </c>
-      <c r="C31" s="71"/>
-      <c r="D31" s="65"/>
-      <c r="E31" s="65"/>
-      <c r="F31" s="65"/>
-      <c r="G31" s="54"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="22">
+      <c r="C31" s="44"/>
+      <c r="D31" s="89"/>
+      <c r="E31" s="89"/>
+      <c r="F31" s="89"/>
+      <c r="G31" s="87"/>
+      <c r="H31" s="103"/>
+      <c r="I31" s="80"/>
+      <c r="J31" s="88">
         <v>18</v>
       </c>
-      <c r="K31" s="64"/>
-      <c r="L31" s="65"/>
-      <c r="M31" s="65"/>
-      <c r="N31" s="65"/>
-      <c r="O31" s="54"/>
-      <c r="P31" s="34"/>
-    </row>
-    <row r="32" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="22">
+      <c r="K31" s="39"/>
+      <c r="L31" s="89"/>
+      <c r="M31" s="89"/>
+      <c r="N31" s="89"/>
+      <c r="O31" s="87"/>
+      <c r="P31" s="103"/>
+      <c r="Q31" s="108"/>
+    </row>
+    <row r="32" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="108"/>
+      <c r="B32" s="88">
         <v>19</v>
       </c>
-      <c r="C32" s="71"/>
-      <c r="D32" s="65"/>
-      <c r="E32" s="65"/>
-      <c r="F32" s="65"/>
-      <c r="G32" s="56"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="22">
+      <c r="C32" s="44"/>
+      <c r="D32" s="89"/>
+      <c r="E32" s="89"/>
+      <c r="F32" s="89"/>
+      <c r="G32" s="92"/>
+      <c r="H32" s="104"/>
+      <c r="I32" s="86"/>
+      <c r="J32" s="88">
         <v>19</v>
       </c>
-      <c r="K32" s="64"/>
-      <c r="L32" s="65"/>
-      <c r="M32" s="65"/>
-      <c r="N32" s="65"/>
-      <c r="O32" s="56"/>
-      <c r="P32" s="35"/>
-    </row>
-    <row r="33" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="22">
+      <c r="K32" s="39"/>
+      <c r="L32" s="89"/>
+      <c r="M32" s="89"/>
+      <c r="N32" s="89"/>
+      <c r="O32" s="92"/>
+      <c r="P32" s="104"/>
+      <c r="Q32" s="108"/>
+    </row>
+    <row r="33" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="108"/>
+      <c r="B33" s="88">
         <v>20</v>
       </c>
-      <c r="C33" s="69"/>
-      <c r="D33" s="69"/>
-      <c r="E33" s="69"/>
-      <c r="F33" s="69"/>
-      <c r="G33" s="54"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="22">
+      <c r="C33" s="43"/>
+      <c r="D33" s="43"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
+      <c r="G33" s="87"/>
+      <c r="H33" s="103"/>
+      <c r="I33" s="80"/>
+      <c r="J33" s="88">
         <v>20</v>
       </c>
-      <c r="K33" s="69"/>
-      <c r="L33" s="69"/>
-      <c r="M33" s="69"/>
-      <c r="N33" s="69"/>
-      <c r="O33" s="54"/>
-      <c r="P33" s="34"/>
-    </row>
-    <row r="34" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="22">
+      <c r="K33" s="43"/>
+      <c r="L33" s="43"/>
+      <c r="M33" s="43"/>
+      <c r="N33" s="43"/>
+      <c r="O33" s="87"/>
+      <c r="P33" s="103"/>
+      <c r="Q33" s="108"/>
+    </row>
+    <row r="34" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="108"/>
+      <c r="B34" s="88">
         <v>21</v>
       </c>
-      <c r="C34" s="69"/>
-      <c r="D34" s="69"/>
-      <c r="E34" s="69"/>
-      <c r="F34" s="69"/>
-      <c r="G34" s="56"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="22">
+      <c r="C34" s="43"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="92"/>
+      <c r="H34" s="103"/>
+      <c r="I34" s="80"/>
+      <c r="J34" s="88">
         <v>21</v>
       </c>
-      <c r="K34" s="69"/>
-      <c r="L34" s="69"/>
-      <c r="M34" s="69"/>
-      <c r="N34" s="69"/>
-      <c r="O34" s="56"/>
-      <c r="P34" s="34"/>
-    </row>
-    <row r="35" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="22">
+      <c r="K34" s="43"/>
+      <c r="L34" s="43"/>
+      <c r="M34" s="43"/>
+      <c r="N34" s="43"/>
+      <c r="O34" s="92"/>
+      <c r="P34" s="103"/>
+      <c r="Q34" s="108"/>
+    </row>
+    <row r="35" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="108"/>
+      <c r="B35" s="88">
         <v>22</v>
       </c>
-      <c r="C35" s="69"/>
-      <c r="D35" s="69"/>
-      <c r="E35" s="69"/>
-      <c r="F35" s="69"/>
-      <c r="G35" s="56"/>
-      <c r="H35" s="36"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="22">
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="92"/>
+      <c r="H35" s="105"/>
+      <c r="I35" s="80"/>
+      <c r="J35" s="88">
         <v>22</v>
       </c>
-      <c r="K35" s="69"/>
-      <c r="L35" s="69"/>
-      <c r="M35" s="69"/>
-      <c r="N35" s="69"/>
-      <c r="O35" s="56"/>
-      <c r="P35" s="36"/>
-    </row>
-    <row r="36" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="22">
+      <c r="K35" s="43"/>
+      <c r="L35" s="43"/>
+      <c r="M35" s="43"/>
+      <c r="N35" s="43"/>
+      <c r="O35" s="92"/>
+      <c r="P35" s="105"/>
+      <c r="Q35" s="108"/>
+    </row>
+    <row r="36" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="108"/>
+      <c r="B36" s="88">
         <v>23</v>
       </c>
-      <c r="C36" s="69"/>
-      <c r="D36" s="69"/>
-      <c r="E36" s="69"/>
-      <c r="F36" s="69"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="36"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="22">
+      <c r="C36" s="43"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="43"/>
+      <c r="F36" s="43"/>
+      <c r="G36" s="92"/>
+      <c r="H36" s="105"/>
+      <c r="I36" s="80"/>
+      <c r="J36" s="88">
         <v>23</v>
       </c>
-      <c r="K36" s="69"/>
-      <c r="L36" s="69"/>
-      <c r="M36" s="69"/>
-      <c r="N36" s="69"/>
-      <c r="O36" s="56"/>
-      <c r="P36" s="36"/>
-    </row>
-    <row r="37" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="22">
+      <c r="K36" s="43"/>
+      <c r="L36" s="43"/>
+      <c r="M36" s="43"/>
+      <c r="N36" s="43"/>
+      <c r="O36" s="92"/>
+      <c r="P36" s="105"/>
+      <c r="Q36" s="108"/>
+    </row>
+    <row r="37" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="108"/>
+      <c r="B37" s="88">
         <v>24</v>
       </c>
-      <c r="C37" s="69"/>
-      <c r="D37" s="69"/>
-      <c r="E37" s="69"/>
-      <c r="F37" s="69"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="36"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="22">
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="92"/>
+      <c r="H37" s="105"/>
+      <c r="I37" s="80"/>
+      <c r="J37" s="88">
         <v>24</v>
       </c>
-      <c r="K37" s="69"/>
-      <c r="L37" s="69"/>
-      <c r="M37" s="69"/>
-      <c r="N37" s="69"/>
-      <c r="O37" s="56"/>
-      <c r="P37" s="36"/>
-    </row>
-    <row r="38" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="22">
+      <c r="K37" s="43"/>
+      <c r="L37" s="43"/>
+      <c r="M37" s="43"/>
+      <c r="N37" s="43"/>
+      <c r="O37" s="92"/>
+      <c r="P37" s="105"/>
+      <c r="Q37" s="108"/>
+    </row>
+    <row r="38" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="108"/>
+      <c r="B38" s="88">
         <v>25</v>
       </c>
-      <c r="C38" s="71"/>
-      <c r="D38" s="65"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="55"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="22">
+      <c r="C38" s="44"/>
+      <c r="D38" s="89"/>
+      <c r="E38" s="89"/>
+      <c r="F38" s="89"/>
+      <c r="G38" s="90"/>
+      <c r="H38" s="105"/>
+      <c r="I38" s="80"/>
+      <c r="J38" s="88">
         <v>25</v>
       </c>
-      <c r="K38" s="64"/>
-      <c r="L38" s="65"/>
-      <c r="M38" s="65"/>
-      <c r="N38" s="65"/>
-      <c r="O38" s="55"/>
-      <c r="P38" s="36"/>
-      <c r="T38" s="37"/>
-    </row>
-    <row r="39" spans="2:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="22">
+      <c r="K38" s="39"/>
+      <c r="L38" s="89"/>
+      <c r="M38" s="89"/>
+      <c r="N38" s="89"/>
+      <c r="O38" s="90"/>
+      <c r="P38" s="105"/>
+      <c r="Q38" s="108"/>
+      <c r="T38" s="17"/>
+    </row>
+    <row r="39" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="108"/>
+      <c r="B39" s="88">
         <v>26</v>
       </c>
-      <c r="C39" s="71"/>
-      <c r="D39" s="65"/>
-      <c r="E39" s="65"/>
-      <c r="F39" s="65"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="36"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="22">
+      <c r="C39" s="44"/>
+      <c r="D39" s="89"/>
+      <c r="E39" s="89"/>
+      <c r="F39" s="89"/>
+      <c r="G39" s="92"/>
+      <c r="H39" s="105"/>
+      <c r="I39" s="86"/>
+      <c r="J39" s="88">
         <v>26</v>
       </c>
-      <c r="K39" s="64"/>
-      <c r="L39" s="65"/>
-      <c r="M39" s="65"/>
-      <c r="N39" s="65"/>
-      <c r="O39" s="56"/>
-      <c r="P39" s="36"/>
-    </row>
-    <row r="40" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="22">
+      <c r="K39" s="39"/>
+      <c r="L39" s="89"/>
+      <c r="M39" s="89"/>
+      <c r="N39" s="89"/>
+      <c r="O39" s="92"/>
+      <c r="P39" s="105"/>
+      <c r="Q39" s="108"/>
+    </row>
+    <row r="40" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="108"/>
+      <c r="B40" s="88">
         <v>27</v>
       </c>
-      <c r="C40" s="71"/>
-      <c r="D40" s="65"/>
-      <c r="E40" s="65"/>
-      <c r="F40" s="65"/>
-      <c r="G40" s="56"/>
-      <c r="H40" s="36"/>
-      <c r="I40" s="21"/>
-      <c r="J40" s="22">
+      <c r="C40" s="44"/>
+      <c r="D40" s="89"/>
+      <c r="E40" s="89"/>
+      <c r="F40" s="89"/>
+      <c r="G40" s="92"/>
+      <c r="H40" s="105"/>
+      <c r="I40" s="86"/>
+      <c r="J40" s="88">
         <v>27</v>
       </c>
-      <c r="K40" s="64"/>
-      <c r="L40" s="65"/>
-      <c r="M40" s="65"/>
-      <c r="N40" s="65"/>
-      <c r="O40" s="56"/>
-      <c r="P40" s="36"/>
-    </row>
-    <row r="41" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="22">
+      <c r="K40" s="39"/>
+      <c r="L40" s="89"/>
+      <c r="M40" s="89"/>
+      <c r="N40" s="89"/>
+      <c r="O40" s="92"/>
+      <c r="P40" s="105"/>
+      <c r="Q40" s="108"/>
+    </row>
+    <row r="41" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="108"/>
+      <c r="B41" s="88">
         <v>28</v>
       </c>
-      <c r="C41" s="65"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="65"/>
-      <c r="G41" s="56"/>
-      <c r="H41" s="36"/>
-      <c r="I41" s="21"/>
-      <c r="J41" s="22">
+      <c r="C41" s="89"/>
+      <c r="D41" s="106"/>
+      <c r="E41" s="106"/>
+      <c r="F41" s="89"/>
+      <c r="G41" s="92"/>
+      <c r="H41" s="105"/>
+      <c r="I41" s="86"/>
+      <c r="J41" s="88">
         <v>28</v>
       </c>
-      <c r="K41" s="65"/>
-      <c r="L41" s="70"/>
-      <c r="M41" s="70"/>
-      <c r="N41" s="65"/>
-      <c r="O41" s="56"/>
-      <c r="P41" s="36"/>
-      <c r="T41" s="29"/>
-    </row>
-    <row r="42" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="22">
+      <c r="K41" s="89"/>
+      <c r="L41" s="106"/>
+      <c r="M41" s="106"/>
+      <c r="N41" s="89"/>
+      <c r="O41" s="92"/>
+      <c r="P41" s="105"/>
+      <c r="Q41" s="108"/>
+      <c r="T41" s="16"/>
+    </row>
+    <row r="42" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="108"/>
+      <c r="B42" s="88">
         <v>29</v>
       </c>
-      <c r="C42" s="65"/>
-      <c r="D42" s="70"/>
-      <c r="E42" s="70"/>
-      <c r="F42" s="65"/>
-      <c r="G42" s="56"/>
-      <c r="H42" s="36"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="22">
+      <c r="C42" s="89"/>
+      <c r="D42" s="106"/>
+      <c r="E42" s="106"/>
+      <c r="F42" s="89"/>
+      <c r="G42" s="92"/>
+      <c r="H42" s="105"/>
+      <c r="I42" s="80"/>
+      <c r="J42" s="88">
         <v>29</v>
       </c>
-      <c r="K42" s="65"/>
-      <c r="L42" s="70"/>
-      <c r="M42" s="70"/>
-      <c r="N42" s="65"/>
-      <c r="O42" s="56"/>
-      <c r="P42" s="36"/>
-      <c r="R42" s="28" t="s">
+      <c r="K42" s="89"/>
+      <c r="L42" s="106"/>
+      <c r="M42" s="106"/>
+      <c r="N42" s="89"/>
+      <c r="O42" s="92"/>
+      <c r="P42" s="105"/>
+      <c r="Q42" s="108"/>
+      <c r="R42" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="T42" s="29"/>
-    </row>
-    <row r="43" spans="2:23" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="22">
+      <c r="T42" s="16"/>
+    </row>
+    <row r="43" spans="1:23" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="108"/>
+      <c r="B43" s="88">
         <v>30</v>
       </c>
-      <c r="C43" s="65"/>
-      <c r="D43" s="65"/>
-      <c r="E43" s="65"/>
-      <c r="F43" s="65"/>
-      <c r="G43" s="56"/>
-      <c r="H43" s="36"/>
-      <c r="I43" s="7"/>
-      <c r="J43" s="22">
+      <c r="C43" s="89"/>
+      <c r="D43" s="89"/>
+      <c r="E43" s="89"/>
+      <c r="F43" s="89"/>
+      <c r="G43" s="92"/>
+      <c r="H43" s="105"/>
+      <c r="I43" s="107"/>
+      <c r="J43" s="88">
         <v>30</v>
       </c>
-      <c r="K43" s="65"/>
-      <c r="L43" s="65"/>
-      <c r="M43" s="65"/>
-      <c r="N43" s="65"/>
-      <c r="O43" s="56"/>
-      <c r="P43" s="36"/>
-      <c r="W43" s="38"/>
-    </row>
-    <row r="44" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="22">
+      <c r="K43" s="89"/>
+      <c r="L43" s="89"/>
+      <c r="M43" s="89"/>
+      <c r="N43" s="89"/>
+      <c r="O43" s="92"/>
+      <c r="P43" s="105"/>
+      <c r="Q43" s="108"/>
+      <c r="W43" s="18"/>
+    </row>
+    <row r="44" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="108"/>
+      <c r="B44" s="88">
         <v>31</v>
       </c>
-      <c r="C44" s="71"/>
-      <c r="D44" s="65"/>
-      <c r="E44" s="65"/>
-      <c r="F44" s="65"/>
-      <c r="G44" s="56"/>
-      <c r="H44" s="36"/>
-      <c r="I44" s="7"/>
-      <c r="J44" s="22">
+      <c r="C44" s="44"/>
+      <c r="D44" s="89"/>
+      <c r="E44" s="89"/>
+      <c r="F44" s="89"/>
+      <c r="G44" s="92"/>
+      <c r="H44" s="105"/>
+      <c r="I44" s="107"/>
+      <c r="J44" s="88">
         <v>31</v>
       </c>
-      <c r="K44" s="64"/>
-      <c r="L44" s="65"/>
-      <c r="M44" s="65"/>
-      <c r="N44" s="65"/>
-      <c r="O44" s="56"/>
-      <c r="P44" s="36"/>
-    </row>
-    <row r="45" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="97"/>
-      <c r="C45" s="98"/>
-      <c r="D45" s="98"/>
-      <c r="E45" s="99"/>
-      <c r="F45" s="68" t="s">
+      <c r="K44" s="39"/>
+      <c r="L44" s="89"/>
+      <c r="M44" s="89"/>
+      <c r="N44" s="89"/>
+      <c r="O44" s="92"/>
+      <c r="P44" s="105"/>
+      <c r="Q44" s="108"/>
+    </row>
+    <row r="45" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="70"/>
+      <c r="C45" s="71"/>
+      <c r="D45" s="71"/>
+      <c r="E45" s="72"/>
+      <c r="F45" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="G45" s="81"/>
-      <c r="H45" s="82"/>
+      <c r="G45" s="52"/>
+      <c r="H45" s="53"/>
       <c r="I45" s="7"/>
-      <c r="J45" s="97"/>
-      <c r="K45" s="98"/>
-      <c r="L45" s="98"/>
-      <c r="M45" s="99"/>
-      <c r="N45" s="68" t="s">
+      <c r="J45" s="70"/>
+      <c r="K45" s="71"/>
+      <c r="L45" s="71"/>
+      <c r="M45" s="72"/>
+      <c r="N45" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="O45" s="81"/>
-      <c r="P45" s="82"/>
-    </row>
-    <row r="46" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="100"/>
-      <c r="C46" s="79"/>
-      <c r="D46" s="79"/>
-      <c r="E46" s="99"/>
-      <c r="F46" s="39" t="s">
+      <c r="O45" s="52"/>
+      <c r="P45" s="53"/>
+    </row>
+    <row r="46" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="73"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
+      <c r="E46" s="72"/>
+      <c r="F46" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G46" s="81"/>
-      <c r="H46" s="82"/>
+      <c r="G46" s="52"/>
+      <c r="H46" s="53"/>
       <c r="I46" s="7"/>
-      <c r="J46" s="100"/>
-      <c r="K46" s="79"/>
-      <c r="L46" s="79"/>
-      <c r="M46" s="99"/>
-      <c r="N46" s="39" t="s">
+      <c r="J46" s="73"/>
+      <c r="K46" s="50"/>
+      <c r="L46" s="50"/>
+      <c r="M46" s="72"/>
+      <c r="N46" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="O46" s="81"/>
-      <c r="P46" s="82"/>
-    </row>
-    <row r="47" spans="2:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="100"/>
-      <c r="C47" s="79"/>
-      <c r="D47" s="79"/>
-      <c r="E47" s="99"/>
-      <c r="F47" s="39" t="s">
+      <c r="O46" s="52"/>
+      <c r="P46" s="53"/>
+    </row>
+    <row r="47" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="73"/>
+      <c r="C47" s="50"/>
+      <c r="D47" s="50"/>
+      <c r="E47" s="72"/>
+      <c r="F47" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G47" s="81"/>
-      <c r="H47" s="82"/>
+      <c r="G47" s="52"/>
+      <c r="H47" s="53"/>
       <c r="I47" s="7"/>
-      <c r="J47" s="100"/>
-      <c r="K47" s="79"/>
-      <c r="L47" s="79"/>
-      <c r="M47" s="99"/>
-      <c r="N47" s="39" t="s">
+      <c r="J47" s="73"/>
+      <c r="K47" s="50"/>
+      <c r="L47" s="50"/>
+      <c r="M47" s="72"/>
+      <c r="N47" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="O47" s="81"/>
-      <c r="P47" s="82"/>
-      <c r="U47" s="29"/>
-    </row>
-    <row r="48" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="100"/>
-      <c r="C48" s="79"/>
-      <c r="D48" s="79"/>
-      <c r="E48" s="99"/>
-      <c r="F48" s="40" t="s">
+      <c r="O47" s="52"/>
+      <c r="P47" s="53"/>
+      <c r="U47" s="16"/>
+    </row>
+    <row r="48" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="73"/>
+      <c r="C48" s="50"/>
+      <c r="D48" s="50"/>
+      <c r="E48" s="72"/>
+      <c r="F48" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="81"/>
-      <c r="H48" s="82"/>
+      <c r="G48" s="52"/>
+      <c r="H48" s="53"/>
       <c r="I48" s="7"/>
-      <c r="J48" s="100"/>
-      <c r="K48" s="79"/>
-      <c r="L48" s="79"/>
-      <c r="M48" s="99"/>
-      <c r="N48" s="40" t="s">
+      <c r="J48" s="73"/>
+      <c r="K48" s="50"/>
+      <c r="L48" s="50"/>
+      <c r="M48" s="72"/>
+      <c r="N48" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="O48" s="81"/>
-      <c r="P48" s="82"/>
-      <c r="U48" s="41"/>
+      <c r="O48" s="52"/>
+      <c r="P48" s="53"/>
+      <c r="U48" s="21"/>
     </row>
     <row r="49" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="42"/>
-      <c r="C49" s="83" t="s">
+      <c r="B49" s="22"/>
+      <c r="C49" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="84"/>
-      <c r="E49" s="84"/>
-      <c r="F49" s="84"/>
-      <c r="G49" s="84"/>
-      <c r="H49" s="85"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="56"/>
       <c r="I49" s="7"/>
-      <c r="J49" s="42"/>
-      <c r="K49" s="83" t="s">
+      <c r="J49" s="22"/>
+      <c r="K49" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="L49" s="84"/>
-      <c r="M49" s="84"/>
-      <c r="N49" s="84"/>
-      <c r="O49" s="84"/>
-      <c r="P49" s="85"/>
+      <c r="L49" s="55"/>
+      <c r="M49" s="55"/>
+      <c r="N49" s="55"/>
+      <c r="O49" s="55"/>
+      <c r="P49" s="56"/>
     </row>
     <row r="50" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="86" t="s">
+      <c r="B50" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="C50" s="79"/>
-      <c r="D50" s="79"/>
-      <c r="E50" s="79"/>
-      <c r="F50" s="79"/>
-      <c r="G50" s="79"/>
-      <c r="H50" s="80"/>
+      <c r="C50" s="50"/>
+      <c r="D50" s="50"/>
+      <c r="E50" s="50"/>
+      <c r="F50" s="50"/>
+      <c r="G50" s="50"/>
+      <c r="H50" s="51"/>
       <c r="I50" s="7"/>
-      <c r="J50" s="86" t="s">
+      <c r="J50" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="K50" s="79"/>
-      <c r="L50" s="79"/>
-      <c r="M50" s="79"/>
-      <c r="N50" s="79"/>
-      <c r="O50" s="79"/>
-      <c r="P50" s="80"/>
+      <c r="K50" s="50"/>
+      <c r="L50" s="50"/>
+      <c r="M50" s="50"/>
+      <c r="N50" s="50"/>
+      <c r="O50" s="50"/>
+      <c r="P50" s="51"/>
     </row>
     <row r="51" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="86" t="s">
+      <c r="B51" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="C51" s="79"/>
-      <c r="D51" s="79"/>
-      <c r="E51" s="79"/>
-      <c r="F51" s="79"/>
-      <c r="G51" s="79"/>
-      <c r="H51" s="80"/>
+      <c r="C51" s="50"/>
+      <c r="D51" s="50"/>
+      <c r="E51" s="50"/>
+      <c r="F51" s="50"/>
+      <c r="G51" s="50"/>
+      <c r="H51" s="51"/>
       <c r="I51" s="9"/>
-      <c r="J51" s="86" t="s">
+      <c r="J51" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="K51" s="79"/>
-      <c r="L51" s="79"/>
-      <c r="M51" s="79"/>
-      <c r="N51" s="79"/>
-      <c r="O51" s="79"/>
-      <c r="P51" s="80"/>
+      <c r="K51" s="50"/>
+      <c r="L51" s="50"/>
+      <c r="M51" s="50"/>
+      <c r="N51" s="50"/>
+      <c r="O51" s="50"/>
+      <c r="P51" s="51"/>
     </row>
     <row r="52" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="86" t="s">
+      <c r="B52" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="C52" s="79"/>
-      <c r="D52" s="79"/>
+      <c r="C52" s="50"/>
+      <c r="D52" s="50"/>
       <c r="E52" s="7"/>
       <c r="F52" s="7"/>
       <c r="G52" s="7"/>
       <c r="H52" s="10"/>
       <c r="I52" s="9"/>
-      <c r="J52" s="86" t="s">
+      <c r="J52" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="K52" s="79"/>
-      <c r="L52" s="79"/>
+      <c r="K52" s="50"/>
+      <c r="L52" s="50"/>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
       <c r="O52" s="7"/>
       <c r="P52" s="10"/>
     </row>
     <row r="53" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="43"/>
+      <c r="B53" s="23"/>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
-      <c r="H53" s="44"/>
+      <c r="H53" s="24"/>
       <c r="I53" s="9"/>
-      <c r="J53" s="43"/>
+      <c r="J53" s="23"/>
       <c r="K53" s="9"/>
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9"/>
       <c r="O53" s="9"/>
-      <c r="P53" s="44"/>
+      <c r="P53" s="24"/>
     </row>
     <row r="54" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="43"/>
+      <c r="B54" s="23"/>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
-      <c r="H54" s="44"/>
+      <c r="H54" s="24"/>
       <c r="I54" s="9"/>
-      <c r="J54" s="43"/>
+      <c r="J54" s="23"/>
       <c r="K54" s="9"/>
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9"/>
       <c r="O54" s="9"/>
-      <c r="P54" s="44"/>
+      <c r="P54" s="24"/>
     </row>
     <row r="55" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="45"/>
-      <c r="C55" s="103"/>
-      <c r="D55" s="104"/>
-      <c r="E55" s="104"/>
-      <c r="F55" s="104"/>
-      <c r="G55" s="104"/>
-      <c r="H55" s="46"/>
+      <c r="B55" s="25"/>
+      <c r="C55" s="58"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="59"/>
+      <c r="F55" s="59"/>
+      <c r="G55" s="59"/>
+      <c r="H55" s="26"/>
       <c r="I55" s="9"/>
-      <c r="J55" s="45"/>
-      <c r="K55" s="103"/>
-      <c r="L55" s="104"/>
-      <c r="M55" s="104"/>
-      <c r="N55" s="104"/>
-      <c r="O55" s="104"/>
-      <c r="P55" s="46"/>
+      <c r="J55" s="25"/>
+      <c r="K55" s="58"/>
+      <c r="L55" s="59"/>
+      <c r="M55" s="59"/>
+      <c r="N55" s="59"/>
+      <c r="O55" s="59"/>
+      <c r="P55" s="26"/>
     </row>
     <row r="56" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="87" t="s">
+      <c r="B56" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="C56" s="79"/>
-      <c r="D56" s="79"/>
-      <c r="E56" s="79"/>
-      <c r="F56" s="79"/>
-      <c r="G56" s="79"/>
-      <c r="H56" s="80"/>
+      <c r="C56" s="50"/>
+      <c r="D56" s="50"/>
+      <c r="E56" s="50"/>
+      <c r="F56" s="50"/>
+      <c r="G56" s="50"/>
+      <c r="H56" s="51"/>
       <c r="I56" s="9"/>
-      <c r="J56" s="87" t="s">
+      <c r="J56" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="K56" s="79"/>
-      <c r="L56" s="79"/>
-      <c r="M56" s="79"/>
-      <c r="N56" s="79"/>
-      <c r="O56" s="79"/>
-      <c r="P56" s="80"/>
+      <c r="K56" s="50"/>
+      <c r="L56" s="50"/>
+      <c r="M56" s="50"/>
+      <c r="N56" s="50"/>
+      <c r="O56" s="50"/>
+      <c r="P56" s="51"/>
     </row>
     <row r="57" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="43" t="s">
+      <c r="B57" s="23" t="s">
         <v>23</v>
       </c>
       <c r="C57" s="9"/>
@@ -2408,9 +2540,9 @@
       <c r="E57" s="9"/>
       <c r="F57" s="9"/>
       <c r="G57" s="9"/>
-      <c r="H57" s="44"/>
+      <c r="H57" s="24"/>
       <c r="I57" s="9"/>
-      <c r="J57" s="43" t="s">
+      <c r="J57" s="23" t="s">
         <v>23</v>
       </c>
       <c r="K57" s="9"/>
@@ -2418,117 +2550,117 @@
       <c r="M57" s="9"/>
       <c r="N57" s="9"/>
       <c r="O57" s="9"/>
-      <c r="P57" s="44"/>
+      <c r="P57" s="24"/>
     </row>
     <row r="58" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="43"/>
+      <c r="B58" s="23"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
-      <c r="H58" s="44"/>
+      <c r="H58" s="24"/>
       <c r="I58" s="9"/>
-      <c r="J58" s="43"/>
+      <c r="J58" s="23"/>
       <c r="K58" s="9"/>
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
-      <c r="P58" s="44"/>
+      <c r="P58" s="24"/>
     </row>
     <row r="59" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="43"/>
+      <c r="B59" s="23"/>
       <c r="C59" s="9"/>
       <c r="D59" s="9"/>
       <c r="E59" s="9"/>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
-      <c r="H59" s="44"/>
+      <c r="H59" s="24"/>
       <c r="I59" s="1"/>
-      <c r="J59" s="43"/>
+      <c r="J59" s="23"/>
       <c r="K59" s="9"/>
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9"/>
       <c r="O59" s="9"/>
-      <c r="P59" s="44"/>
+      <c r="P59" s="24"/>
     </row>
     <row r="60" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="43"/>
+      <c r="B60" s="23"/>
       <c r="C60" s="9"/>
       <c r="D60" s="9"/>
       <c r="E60" s="9"/>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
-      <c r="H60" s="44"/>
+      <c r="H60" s="24"/>
       <c r="I60" s="9"/>
-      <c r="J60" s="43"/>
+      <c r="J60" s="23"/>
       <c r="K60" s="9"/>
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9"/>
       <c r="O60" s="9"/>
-      <c r="P60" s="44"/>
+      <c r="P60" s="24"/>
     </row>
     <row r="61" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="47"/>
-      <c r="C61" s="76"/>
-      <c r="D61" s="77"/>
-      <c r="E61" s="77"/>
-      <c r="F61" s="77"/>
-      <c r="G61" s="77"/>
-      <c r="H61" s="48"/>
+      <c r="B61" s="27"/>
+      <c r="C61" s="47"/>
+      <c r="D61" s="48"/>
+      <c r="E61" s="48"/>
+      <c r="F61" s="48"/>
+      <c r="G61" s="48"/>
+      <c r="H61" s="28"/>
       <c r="I61" s="9"/>
-      <c r="J61" s="47"/>
-      <c r="K61" s="101"/>
-      <c r="L61" s="102"/>
-      <c r="M61" s="102"/>
-      <c r="N61" s="102"/>
-      <c r="O61" s="102"/>
-      <c r="P61" s="48"/>
+      <c r="J61" s="27"/>
+      <c r="K61" s="74"/>
+      <c r="L61" s="75"/>
+      <c r="M61" s="75"/>
+      <c r="N61" s="75"/>
+      <c r="O61" s="75"/>
+      <c r="P61" s="28"/>
     </row>
     <row r="62" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="78"/>
-      <c r="C62" s="79"/>
-      <c r="D62" s="79"/>
-      <c r="E62" s="79"/>
-      <c r="F62" s="79"/>
-      <c r="G62" s="79"/>
-      <c r="H62" s="80"/>
-      <c r="I62" s="49"/>
-      <c r="J62" s="78"/>
-      <c r="K62" s="79"/>
-      <c r="L62" s="79"/>
-      <c r="M62" s="79"/>
-      <c r="N62" s="79"/>
-      <c r="O62" s="79"/>
-      <c r="P62" s="80"/>
+      <c r="B62" s="49"/>
+      <c r="C62" s="50"/>
+      <c r="D62" s="50"/>
+      <c r="E62" s="50"/>
+      <c r="F62" s="50"/>
+      <c r="G62" s="50"/>
+      <c r="H62" s="51"/>
+      <c r="I62" s="29"/>
+      <c r="J62" s="49"/>
+      <c r="K62" s="50"/>
+      <c r="L62" s="50"/>
+      <c r="M62" s="50"/>
+      <c r="N62" s="50"/>
+      <c r="O62" s="50"/>
+      <c r="P62" s="51"/>
     </row>
     <row r="63" spans="2:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="50"/>
-      <c r="C63" s="51"/>
-      <c r="D63" s="51"/>
-      <c r="E63" s="51"/>
-      <c r="F63" s="51"/>
-      <c r="G63" s="51"/>
-      <c r="H63" s="52"/>
-      <c r="J63" s="50"/>
-      <c r="K63" s="51"/>
-      <c r="L63" s="51"/>
-      <c r="M63" s="51"/>
-      <c r="N63" s="51"/>
-      <c r="O63" s="51"/>
-      <c r="P63" s="52"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="31"/>
+      <c r="F63" s="31"/>
+      <c r="G63" s="31"/>
+      <c r="H63" s="32"/>
+      <c r="J63" s="30"/>
+      <c r="K63" s="31"/>
+      <c r="L63" s="31"/>
+      <c r="M63" s="31"/>
+      <c r="N63" s="31"/>
+      <c r="O63" s="31"/>
+      <c r="P63" s="32"/>
     </row>
     <row r="64" spans="2:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="49"/>
-      <c r="C64" s="49"/>
-      <c r="D64" s="49"/>
-      <c r="E64" s="49"/>
-      <c r="F64" s="49"/>
-      <c r="G64" s="49"/>
-      <c r="H64" s="49"/>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="E64" s="29"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="29"/>
     </row>
     <row r="65" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="66" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>